<commit_message>
chore(doc): retire les colonnes Forfait jour et Tickets restaurant du template Kostango
</commit_message>
<xml_diff>
--- a/doc/template_utilisateurs_kostango.xlsx
+++ b/doc/template_utilisateurs_kostango.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -433,10 +433,8 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,20 +505,10 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Forfait jour</t>
+          <t>Agence d'intérim</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Tickets restaurant</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Agence d'intérim</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>valideur N+1</t>
         </is>

</xml_diff>

<commit_message>
feat(users): ajoute Service et Rôle applicatif à l'import Kostango
- lit les colonnes "Service" (get_or_create) et "Rôle" (validé contre les
  rôles applicatifs existants, employee par défaut) dans import_kostango
- synchronise service et role sur les utilisateurs déjà existants lors d'une
  ré-importation (comme les autres champs)
- ajoute les colonnes correspondantes au template xlsx
</commit_message>
<xml_diff>
--- a/doc/template_utilisateurs_kostango.xlsx
+++ b/doc/template_utilisateurs_kostango.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -433,8 +433,10 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,30 +487,40 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Poste</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Type contrat</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Coefficient</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Rôle</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Agence d'intérim</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>valideur N+1</t>
         </is>

</xml_diff>

<commit_message>
fix(users): résout le N+1 de l'import Kostango par matricule plutôt que par nom
Deux personnes peuvent porter le même prénom/nom ; la colonne "valideur N+1"
(recherche par nom complet) est remplacée par "Matricule N+1" (référence
directe et sans ambiguïté). Templates et exemple xlsx mis à jour en conséquence.
</commit_message>
<xml_diff>
--- a/doc/template_utilisateurs_kostango.xlsx
+++ b/doc/template_utilisateurs_kostango.xlsx
@@ -436,7 +436,7 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,7 +522,7 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>valideur N+1</t>
+          <t>Matricule N+1</t>
         </is>
       </c>
     </row>

</xml_diff>